<commit_message>
feat: update cards and battle presentation
</commit_message>
<xml_diff>
--- a/DataTables/Datas/Character/#UpgradeOptions.xlsx
+++ b/DataTables/Datas/Character/#UpgradeOptions.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,20 +439,30 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>IsCommon</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Rarity</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Prerequisite</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Effects</t>
         </is>
@@ -476,25 +486,35 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CharacterEnum</t>
+          <t>CharacterEnum?</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>RarityEnum</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>string?</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>(list#sep=;),(UpgradeEffect#sep=,)</t>
         </is>
@@ -525,25 +545,35 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>从属角色</t>
+          <t>从属角色(公共选项留空)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>是否进入所有角色的公共池</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>构筑主题；副选项必须与前置主题一致</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>升级文本</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>稀有度</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>前置升级选项(填Id,空=无)</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>实装效果(多态;分隔,空=暂无)</t>
         </is>
@@ -552,133 +582,780 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>UP_Rocket_001</t>
+          <t>UP_Common_001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>强化爆破</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Rocket</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>「爆破」造成的伤害 +5</t>
-        </is>
+          <t>强健根基</t>
+        </is>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>最大生命 +6</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>ModifyCardStat,Rocket001,Damage,5</t>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>ModifyUnitStat,MaxHp,6,Self</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>UP_Rocket_002</t>
+          <t>UP_Common_002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>连锁爆破</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Rocket</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>「爆破」改为对全体敌人造成伤害</t>
-        </is>
+          <t>战斗专注</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>UP_Rocket_001</t>
+          <t>战斗开始时获得 1 点力量</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>ModifyCardFlag,Rocket001,IsAoe,true</t>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>GrantBuff,Strength,1,Self</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>UP_Irene_001</t>
+          <t>UP_Common_003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>凝神</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>战斗开始时获得 2 点力量</t>
-        </is>
+          <t>灵巧身法</t>
+        </is>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>战斗开始时获得 1 点敏捷</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>GrantBuff,Strength,2,Self</t>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>GrantBuff,Dexterity,1,Self</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
+          <t>UP_Rocket_001</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>强化挥砍</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Rocket</t>
+        </is>
+      </c>
+      <c r="E8" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>DirectAttack</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>「挥砍」造成的伤害 +5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Rocket001,Damage,5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UP_Rocket_002</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>横扫挥砍</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Rocket</t>
+        </is>
+      </c>
+      <c r="E9" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>DirectAttack</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>「挥砍」改为对全体敌人造成伤害</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>UP_Rocket_001</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>ModifyCardFlag,Rocket001,IsAoe,true</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>UP_Rocket_003</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>复合装甲</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Rocket</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Armor</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>所有护甲牌的护甲 +2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,All,Defense,2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>UP_Rocket_004</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>战线加固</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Rocket</t>
+        </is>
+      </c>
+      <c r="E11" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Armor</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>「举盾」「装甲齐射」「阵线加固」「应急装甲」「区域装甲」「推进阵线」的护甲额外 +2</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>UP_Rocket_003</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Rocket005,Defense,2;ModifyCardStat,Rocket011,Defense,2;ModifyCardStat,Rocket012,Defense,2;ModifyCardStat,Rocket016,Defense,2;ModifyCardStat,Rocket019,Defense,2;ModifyCardStat,Rocket020,Defense,2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>UP_Rocket_005</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>过载弹头</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Rocket</t>
+        </is>
+      </c>
+      <c r="E12" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Overload</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>「超载火炮」「震荡冲击」造成的伤害 +3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Rocket004,Damage,3;ModifyCardStat,Rocket017,Damage,3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>UP_Rocket_006</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>临界超载</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Rocket</t>
+        </is>
+      </c>
+      <c r="E13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Overload</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>「超载火炮」「震荡冲击」造成的伤害额外 +4</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>UP_Rocket_005</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Rocket004,Damage,4;ModifyCardStat,Rocket017,Damage,4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>UP_Irene_001</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>凝神</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>战斗开始时获得 2 点力量</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>GrantBuff,Strength,2,Self</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UP_Irene_002</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>咏唱增幅</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>所有执行牌造成的伤害 +2</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,CardType:Execution,Damage,2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>UP_Irene_003</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>长线蓄能</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E16" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>所有执行牌造成的伤害额外 +3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>UP_Irene_002</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,CardType:Execution,Damage,3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UP_Irene_004</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>雷云导体</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E17" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>「连锁闪电」造成的伤害 +4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Irene009,Damage,4</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>UP_Irene_005</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>风暴共鸣</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E18" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>「连锁闪电」造成的伤害额外 +6；「终焉倒数」造成的伤害 +4</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>UP_Irene_004</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Irene009,Damage,6;ModifyCardStat,Irene020,Damage,4</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
           <t>UP_Zhouzhou_001</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>坚守</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Zhouzhou</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E19" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>最大生命 +8</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>ModifyUnitStat,MaxHp,8,Self</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>UP_Zhouzhou_002</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>流动掩护</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Zhouzhou</t>
+        </is>
+      </c>
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>「挽袖同行」「游身」提供的护甲 +2</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Zhouzhou005,Defense,2;ModifyCardStat,Zhouzhou007,Defense,2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UP_Zhouzhou_003</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>无痕折返</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Zhouzhou</t>
+        </is>
+      </c>
+      <c r="E21" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>「挽袖同行」「游身」提供的护甲额外 +2</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>UP_Zhouzhou_002</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Zhouzhou005,Defense,2;ModifyCardStat,Zhouzhou007,Defense,2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>UP_Zhouzhou_004</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>飞刃随行</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Zhouzhou</t>
+        </is>
+      </c>
+      <c r="E22" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>「飞刀」造成的伤害 +2</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Extra001,Damage,2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>UP_Zhouzhou_005</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>连步追刃</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Zhouzhou</t>
+        </is>
+      </c>
+      <c r="E23" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>「飞刀」造成的伤害额外 +2；「钩锁」造成的伤害 +2</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>UP_Zhouzhou_004</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>ModifyCardStat,Extra001,Damage,2;ModifyCardStat,Zhouzhou011,Damage,2</t>
         </is>
       </c>
     </row>

</xml_diff>